<commit_message>
feat: verify rule CG0266 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000153/negative/01/data/unit-test-coreid-CG0266-negative 1.xlsx
+++ b/rules/CORE-000153/negative/01/data/unit-test-coreid-CG0266-negative 1.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -88,6 +94,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -529,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,6 +571,210 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TSVCDVER</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TSVCDREF</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TSVCDVER</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TSVCDREF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>21</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TSVCDVER</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2019-03-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TSVCDREF</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>46</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TSVCDVER</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ts.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>46</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TSVCDREF</t>
         </is>
       </c>
     </row>
@@ -848,12 +1062,8 @@
           <t>C49487</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>2020-03-27</t>
         </is>
@@ -893,7 +1103,8 @@
           <t>C49487</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>2020-03-27</t>
         </is>
@@ -1433,7 +1644,8 @@
           <t>26929004</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>2019-03-01</t>
         </is>
@@ -2338,7 +2550,8 @@
           <t>C98388</t>
         </is>
       </c>
-      <c r="K46" s="4" t="inlineStr">
+      <c r="J46" s="6" t="n"/>
+      <c r="K46" s="5" t="inlineStr">
         <is>
           <t>2020-03-27</t>
         </is>

</xml_diff>